<commit_message>
Mise à jour page Seuils
</commit_message>
<xml_diff>
--- a/prix/prix.xlsx
+++ b/prix/prix.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\seuils\prix\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\seuils\prix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1E7BF46-CA29-461B-AC3D-B823C119F236}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52A754F1-C062-44F0-A74D-1BB30B5F4A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6E95DC93-531D-460D-9A06-44397A8920D7}"/>
+    <workbookView xWindow="23124" yWindow="12" windowWidth="19116" windowHeight="10884" xr2:uid="{6E95DC93-531D-460D-9A06-44397A8920D7}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="139">
   <si>
     <t>path</t>
   </si>
@@ -54,6 +54,405 @@
   </si>
   <si>
     <t>disponible</t>
+  </si>
+  <si>
+    <t>79306703</t>
+  </si>
+  <si>
+    <t>79306704</t>
+  </si>
+  <si>
+    <t>79306705</t>
+  </si>
+  <si>
+    <t>79306706</t>
+  </si>
+  <si>
+    <t>79306707</t>
+  </si>
+  <si>
+    <t>79306708</t>
+  </si>
+  <si>
+    <t>79306709</t>
+  </si>
+  <si>
+    <t>79306711</t>
+  </si>
+  <si>
+    <t>79306713</t>
+  </si>
+  <si>
+    <t>79306715</t>
+  </si>
+  <si>
+    <t>79306716</t>
+  </si>
+  <si>
+    <t>79306717</t>
+  </si>
+  <si>
+    <t>79306718</t>
+  </si>
+  <si>
+    <t>79306719</t>
+  </si>
+  <si>
+    <t>79306729</t>
+  </si>
+  <si>
+    <t>79306730</t>
+  </si>
+  <si>
+    <t>79306731</t>
+  </si>
+  <si>
+    <t>79306732</t>
+  </si>
+  <si>
+    <t>79306733</t>
+  </si>
+  <si>
+    <t>79306735</t>
+  </si>
+  <si>
+    <t>79306736</t>
+  </si>
+  <si>
+    <t>79306738</t>
+  </si>
+  <si>
+    <t>79306740</t>
+  </si>
+  <si>
+    <t>79306742</t>
+  </si>
+  <si>
+    <t>79306743</t>
+  </si>
+  <si>
+    <t>79306744</t>
+  </si>
+  <si>
+    <t>79306745</t>
+  </si>
+  <si>
+    <t>79306746</t>
+  </si>
+  <si>
+    <t>79306747</t>
+  </si>
+  <si>
+    <t>79306750</t>
+  </si>
+  <si>
+    <t>79306751</t>
+  </si>
+  <si>
+    <t>79306752</t>
+  </si>
+  <si>
+    <t>79306753</t>
+  </si>
+  <si>
+    <t>79306754</t>
+  </si>
+  <si>
+    <t>79306755</t>
+  </si>
+  <si>
+    <t>79306756</t>
+  </si>
+  <si>
+    <t>79306757</t>
+  </si>
+  <si>
+    <t>79306758</t>
+  </si>
+  <si>
+    <t>79306759</t>
+  </si>
+  <si>
+    <t>79306760</t>
+  </si>
+  <si>
+    <t>79306761</t>
+  </si>
+  <si>
+    <t>79306762</t>
+  </si>
+  <si>
+    <t>79306769</t>
+  </si>
+  <si>
+    <t>79306770</t>
+  </si>
+  <si>
+    <t>79306771</t>
+  </si>
+  <si>
+    <t>79306772</t>
+  </si>
+  <si>
+    <t>79306773</t>
+  </si>
+  <si>
+    <t>79306774</t>
+  </si>
+  <si>
+    <t>79306775</t>
+  </si>
+  <si>
+    <t>79306777</t>
+  </si>
+  <si>
+    <t>79306778</t>
+  </si>
+  <si>
+    <t>79306779</t>
+  </si>
+  <si>
+    <t>79306780</t>
+  </si>
+  <si>
+    <t>79306781</t>
+  </si>
+  <si>
+    <t>79306782</t>
+  </si>
+  <si>
+    <t>79306783</t>
+  </si>
+  <si>
+    <t>79306784</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 18cm 100cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 18cm 110cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 18cm 120cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 18cm 130cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 18cm 140cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 18cm 150cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 18cm 160cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 18cm 170cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 18cm 180cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 22cm 100cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 22cm 110cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 22cm 120cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 22cm 130cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 22cm 140cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 22cm 150cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 22cm 160cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 22cm 170cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 22cm 180cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 22cm 190cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 25cm 100cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 25cm 110cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 25cm 120cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 25cm 130cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 25cm 140cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 25cm 150cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 25cm 160cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 25cm 170cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 28cm 100cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 28cm 110cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 28cm 120cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 28cm 130cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 28cm 140cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 28cm 150cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 28cm 160cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 28cm 170cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 28cm 180cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 28cm 190cm</t>
+  </si>
+  <si>
+    <t>50cm</t>
+  </si>
+  <si>
+    <t>60cm</t>
+  </si>
+  <si>
+    <t>70cm</t>
+  </si>
+  <si>
+    <t>80cm</t>
+  </si>
+  <si>
+    <t>90cm</t>
+  </si>
+  <si>
+    <t>100cm</t>
+  </si>
+  <si>
+    <t>110cm</t>
+  </si>
+  <si>
+    <t>120cm</t>
+  </si>
+  <si>
+    <t>130cm</t>
+  </si>
+  <si>
+    <t>140cm</t>
+  </si>
+  <si>
+    <t>150cm</t>
+  </si>
+  <si>
+    <t>160cm</t>
+  </si>
+  <si>
+    <t>170cm</t>
+  </si>
+  <si>
+    <t>180cm</t>
+  </si>
+  <si>
+    <t>190cm</t>
+  </si>
+  <si>
+    <t>galerie/seuils-18.png</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 18cm 50cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 18cm 60cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 18cm 70cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 18cm 80cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 18cm 90cm</t>
+  </si>
+  <si>
+    <t>galerie/seuils-22.png</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 22cm 50cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 22cm 60cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 22cm 70cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 22cm 80cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 22cm 90cm</t>
+  </si>
+  <si>
+    <t>galerie/seuils-25.png</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 25cm 50cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 25cm 60cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 25cm 70cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 25cm 80cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 25cm 90cm</t>
+  </si>
+  <si>
+    <t>galerie/seuils-28.png</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 28cm 50cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 28cm 60cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 28cm 70cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 28cm 80cm</t>
+  </si>
+  <si>
+    <t>Seuil PT 5cm 28cm 90cm</t>
   </si>
 </sst>
 </file>
@@ -129,7 +528,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -156,16 +555,22 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -505,7 +910,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="51.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="52.21875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5546875" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="28.109375" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.6640625" style="3" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10" style="4" bestFit="1" customWidth="1"/>
@@ -520,7 +925,7 @@
       <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="7" t="s">
@@ -535,373 +940,1144 @@
       <c r="G1" s="2"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="5"/>
-      <c r="B2" s="9"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="10"/>
+      <c r="A2" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D2" s="14">
+        <v>25.33</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="15">
+        <v>6</v>
+      </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="5"/>
-      <c r="B3" s="9"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="10"/>
+      <c r="A3" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D3" s="14">
+        <v>30.38</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="15">
+        <v>14</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="5"/>
-      <c r="B4" s="9"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="10"/>
+      <c r="A4" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D4" s="14">
+        <v>35.450000000000003</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="15">
+        <v>8</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="5"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="10"/>
+      <c r="A5" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D5" s="14">
+        <v>40.51</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="15">
+        <v>7</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="5"/>
-      <c r="B6" s="9"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="10"/>
+      <c r="A6" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D6" s="14">
+        <v>45.58</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="15">
+        <v>11</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="5"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="10"/>
+      <c r="A7" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D7" s="14">
+        <v>50.64</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="15">
+        <v>7</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="5"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="10"/>
+      <c r="A8" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D8" s="14">
+        <v>55.71</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="15">
+        <v>6</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="5"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="10"/>
+      <c r="A9" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D9" s="14">
+        <v>60.77</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="15">
+        <v>11</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="5"/>
-      <c r="B10" s="9"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="10"/>
+      <c r="A10" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D10" s="14">
+        <v>65.84</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" s="15">
+        <v>9</v>
+      </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="5"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="10"/>
+      <c r="A11" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D11" s="14">
+        <v>70.89</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" s="15">
+        <v>9</v>
+      </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="5"/>
-      <c r="B12" s="9"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="10"/>
+      <c r="A12" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D12" s="14">
+        <v>75.959999999999994</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" s="15">
+        <v>6</v>
+      </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="5"/>
-      <c r="B13" s="9"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="10"/>
+      <c r="A13" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D13" s="14">
+        <v>81.02</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F13" s="15">
+        <v>7</v>
+      </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="5"/>
-      <c r="B14" s="9"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="10"/>
+      <c r="A14" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D14" s="14">
+        <v>86.09</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="F14" s="15">
+        <v>5</v>
+      </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="5"/>
-      <c r="B15" s="9"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="10"/>
+      <c r="A15" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D15" s="14">
+        <v>91.15</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F15" s="15">
+        <v>0</v>
+      </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="5"/>
-      <c r="B16" s="9"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="10"/>
+      <c r="A16" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D16" s="14">
+        <v>30.95</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F16" s="15">
+        <v>12</v>
+      </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="5"/>
+      <c r="A17" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D17" s="14">
+        <v>37.130000000000003</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F17" s="15">
+        <v>6</v>
+      </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="5"/>
+      <c r="A18" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D18" s="14">
+        <v>43.33</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="F18" s="15">
+        <v>6</v>
+      </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="5"/>
-      <c r="B19" s="9"/>
-      <c r="C19" s="5"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="5"/>
+      <c r="A19" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D19" s="14">
+        <v>49.51</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F19" s="15">
+        <v>5</v>
+      </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="5"/>
+      <c r="A20" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D20" s="14">
+        <v>55.71</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="F20" s="15">
+        <v>5</v>
+      </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="5"/>
+      <c r="A21" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D21" s="14">
+        <v>61.89</v>
+      </c>
+      <c r="E21" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="F21" s="15">
+        <v>4</v>
+      </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="5"/>
-      <c r="C22" s="5"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="5"/>
+      <c r="A22" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D22" s="14">
+        <v>68.09</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="F22" s="15">
+        <v>11</v>
+      </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="5"/>
-      <c r="C23" s="5"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="5"/>
+      <c r="A23" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D23" s="14">
+        <v>74.27</v>
+      </c>
+      <c r="E23" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="F23" s="15">
+        <v>10</v>
+      </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="5"/>
-      <c r="C24" s="5"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="5"/>
+      <c r="A24" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D24" s="14">
+        <v>80.47</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="F24" s="15">
+        <v>12</v>
+      </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="5"/>
-      <c r="C25" s="5"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="5"/>
+      <c r="A25" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D25" s="14">
+        <v>86.65</v>
+      </c>
+      <c r="E25" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="F25" s="15">
+        <v>6</v>
+      </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="5"/>
-      <c r="C26" s="5"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="5"/>
+      <c r="A26" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D26" s="14">
+        <v>92.84</v>
+      </c>
+      <c r="E26" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F26" s="15">
+        <v>6</v>
+      </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="5"/>
-      <c r="C27" s="5"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="5"/>
+      <c r="A27" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D27" s="14">
+        <v>99.03</v>
+      </c>
+      <c r="E27" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="F27" s="15">
+        <v>10</v>
+      </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="5"/>
-      <c r="C28" s="5"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="5"/>
+      <c r="A28" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D28" s="14">
+        <v>105.22</v>
+      </c>
+      <c r="E28" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="F28" s="15">
+        <v>5</v>
+      </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="5"/>
-      <c r="C29" s="5"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="5"/>
+      <c r="A29" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D29" s="14">
+        <v>111.4</v>
+      </c>
+      <c r="E29" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="F29" s="15">
+        <v>0</v>
+      </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="5"/>
-      <c r="C30" s="5"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="5"/>
+      <c r="A30" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B30" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D30" s="14">
+        <v>117.6</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="F30" s="15">
+        <v>0</v>
+      </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="5"/>
-      <c r="C31" s="5"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="5"/>
+      <c r="A31" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B31" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D31" s="14">
+        <v>35.17</v>
+      </c>
+      <c r="E31" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="F31" s="15">
+        <v>6</v>
+      </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="5"/>
-      <c r="C32" s="5"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="5"/>
+      <c r="A32" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B32" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D32" s="14">
+        <v>42.2</v>
+      </c>
+      <c r="E32" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="F32" s="15">
+        <v>4</v>
+      </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="5"/>
-      <c r="C33" s="5"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="5"/>
+      <c r="A33" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B33" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D33" s="14">
+        <v>49.25</v>
+      </c>
+      <c r="E33" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="F33" s="15">
+        <v>8</v>
+      </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="5"/>
-      <c r="C34" s="5"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="5"/>
+      <c r="A34" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B34" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D34" s="14">
+        <v>56.27</v>
+      </c>
+      <c r="E34" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F34" s="15">
+        <v>8</v>
+      </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="5"/>
-      <c r="C35" s="5"/>
-      <c r="E35" s="2"/>
-      <c r="F35" s="5"/>
+      <c r="A35" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B35" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D35" s="14">
+        <v>63.31</v>
+      </c>
+      <c r="E35" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="F35" s="15">
+        <v>5</v>
+      </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="5"/>
-      <c r="C36" s="5"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="5"/>
+      <c r="A36" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B36" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D36" s="14">
+        <v>70.34</v>
+      </c>
+      <c r="E36" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="F36" s="15">
+        <v>10</v>
+      </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="5"/>
-      <c r="C37" s="5"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="5"/>
+      <c r="A37" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B37" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D37" s="14">
+        <v>77.38</v>
+      </c>
+      <c r="E37" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="F37" s="15">
+        <v>9</v>
+      </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="5"/>
-      <c r="C38" s="5"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="5"/>
+      <c r="A38" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B38" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D38" s="14">
+        <v>84.4</v>
+      </c>
+      <c r="E38" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="F38" s="15">
+        <v>6</v>
+      </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="5"/>
-      <c r="C39" s="5"/>
-      <c r="E39" s="2"/>
-      <c r="F39" s="5"/>
+      <c r="A39" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B39" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D39" s="14">
+        <v>91.44</v>
+      </c>
+      <c r="E39" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="F39" s="15">
+        <v>9</v>
+      </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="5"/>
-      <c r="C40" s="5"/>
-      <c r="E40" s="2"/>
-      <c r="F40" s="5"/>
+      <c r="A40" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B40" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D40" s="14">
+        <v>98.47</v>
+      </c>
+      <c r="E40" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="F40" s="15">
+        <v>5</v>
+      </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="5"/>
-      <c r="C41" s="5"/>
-      <c r="E41" s="2"/>
-      <c r="F41" s="5"/>
+      <c r="A41" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B41" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D41" s="14">
+        <v>105.51</v>
+      </c>
+      <c r="E41" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="F41" s="15">
+        <v>8</v>
+      </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="5"/>
-      <c r="C42" s="5"/>
-      <c r="E42" s="2"/>
-      <c r="F42" s="5"/>
+      <c r="A42" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B42" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D42" s="14">
+        <v>112.53</v>
+      </c>
+      <c r="E42" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="F42" s="15">
+        <v>4</v>
+      </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" s="5"/>
-      <c r="C43" s="5"/>
-      <c r="E43" s="2"/>
-      <c r="F43" s="5"/>
+      <c r="A43" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B43" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D43" s="14">
+        <v>119.57</v>
+      </c>
+      <c r="E43" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="F43" s="15">
+        <v>5</v>
+      </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" s="5"/>
-      <c r="C44" s="5"/>
-      <c r="E44" s="2"/>
-      <c r="F44" s="5"/>
+      <c r="A44" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B44" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D44" s="14">
+        <v>39.39</v>
+      </c>
+      <c r="E44" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="F44" s="15">
+        <v>1</v>
+      </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45" s="5"/>
-      <c r="C45" s="5"/>
-      <c r="E45" s="2"/>
-      <c r="F45" s="5"/>
+      <c r="A45" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B45" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D45" s="14">
+        <v>47.26</v>
+      </c>
+      <c r="E45" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="F45" s="15">
+        <v>5</v>
+      </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" s="5"/>
-      <c r="C46" s="5"/>
-      <c r="E46" s="2"/>
-      <c r="F46" s="5"/>
+      <c r="A46" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B46" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D46" s="14">
+        <v>57.06</v>
+      </c>
+      <c r="E46" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="F46" s="15">
+        <v>6</v>
+      </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="5"/>
-      <c r="C47" s="5"/>
-      <c r="E47" s="2"/>
-      <c r="F47" s="5"/>
+      <c r="A47" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B47" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D47" s="14">
+        <v>63.02</v>
+      </c>
+      <c r="E47" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="F47" s="15">
+        <v>10</v>
+      </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="5"/>
-      <c r="C48" s="5"/>
-      <c r="E48" s="2"/>
-      <c r="F48" s="5"/>
+      <c r="A48" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B48" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D48" s="14">
+        <v>70.89</v>
+      </c>
+      <c r="E48" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="F48" s="15">
+        <v>4</v>
+      </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="5"/>
-      <c r="C49" s="5"/>
-      <c r="E49" s="2"/>
-      <c r="F49" s="5"/>
+      <c r="A49" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B49" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D49" s="14">
+        <v>81.52</v>
+      </c>
+      <c r="E49" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="F49" s="15">
+        <v>6</v>
+      </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" s="5"/>
-      <c r="C50" s="5"/>
-      <c r="E50" s="2"/>
-      <c r="F50" s="5"/>
+      <c r="A50" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B50" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D50" s="14">
+        <v>86.65</v>
+      </c>
+      <c r="E50" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F50" s="15">
+        <v>7</v>
+      </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51" s="5"/>
-      <c r="C51" s="5"/>
-      <c r="E51" s="2"/>
-      <c r="F51" s="5"/>
+      <c r="A51" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B51" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D51" s="14">
+        <v>94.53</v>
+      </c>
+      <c r="E51" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="F51" s="15">
+        <v>10</v>
+      </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" s="5"/>
-      <c r="C52" s="5"/>
-      <c r="E52" s="2"/>
-      <c r="F52" s="5"/>
+      <c r="A52" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B52" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D52" s="14">
+        <v>102.4</v>
+      </c>
+      <c r="E52" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="F52" s="15">
+        <v>6</v>
+      </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="5"/>
-      <c r="B53" s="9"/>
-      <c r="C53" s="5"/>
-      <c r="E53" s="2"/>
-      <c r="F53" s="5"/>
+      <c r="A53" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B53" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D53" s="14">
+        <v>110.28</v>
+      </c>
+      <c r="E53" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="F53" s="15">
+        <v>3</v>
+      </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A54" s="5"/>
-      <c r="C54" s="5"/>
-      <c r="E54" s="2"/>
-      <c r="F54" s="5"/>
+      <c r="A54" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B54" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D54" s="14">
+        <v>122.28</v>
+      </c>
+      <c r="E54" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="F54" s="15">
+        <v>1</v>
+      </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" s="5"/>
-      <c r="B55" s="9"/>
-      <c r="C55" s="5"/>
-      <c r="E55" s="2"/>
-      <c r="F55" s="5"/>
+      <c r="A55" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B55" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D55" s="14">
+        <v>130.43</v>
+      </c>
+      <c r="E55" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="F55" s="15">
+        <v>0</v>
+      </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="5"/>
-      <c r="C56" s="5"/>
-      <c r="E56" s="2"/>
-      <c r="F56" s="5"/>
+      <c r="A56" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B56" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D56" s="14">
+        <v>138.58000000000001</v>
+      </c>
+      <c r="E56" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="F56" s="15">
+        <v>1</v>
+      </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="5"/>
+      <c r="A57" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B57" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D57" s="14">
+        <v>146.72</v>
+      </c>
+      <c r="E57" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="F57" s="15">
+        <v>-5</v>
+      </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="5"/>
+      <c r="A58" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B58" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D58" s="14">
+        <v>154.88</v>
+      </c>
+      <c r="E58" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="F58" s="15">
+        <v>0</v>
+      </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="5"/>
@@ -941,7 +2117,7 @@
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" s="5"/>
-      <c r="G71" s="13"/>
+      <c r="G71" s="11"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" s="5"/>

</xml_diff>